<commit_message>
validacion de calibre de los cables y nuevo reporte
</commit_message>
<xml_diff>
--- a/Program/Datos/DB/datos_manuales.xlsx
+++ b/Program/Datos/DB/datos_manuales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mhoyosme\Desktop\Proyecto\Program\Datos\DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061B74AA-565A-4D2F-8A4A-C832BF1F624B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DA7CF08-90CD-4F86-8DCA-0DFF0117922F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CD6D87B3-3E85-4D9D-BFF0-D4E802493E81}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CD6D87B3-3E85-4D9D-BFF0-D4E802493E81}"/>
   </bookViews>
   <sheets>
     <sheet name="info_nodo" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="196">
   <si>
     <t>75.0</t>
   </si>
@@ -89,12 +89,6 @@
     <t>NM1-125S/3300</t>
   </si>
   <si>
-    <t>Breaker Rect 1</t>
-  </si>
-  <si>
-    <t>Breaker Rect 2</t>
-  </si>
-  <si>
     <t>corriente</t>
   </si>
   <si>
@@ -624,6 +618,15 @@
   </si>
   <si>
     <t>maximo_racks</t>
+  </si>
+  <si>
+    <t>Breaker Rect1</t>
+  </si>
+  <si>
+    <t>Breaker Rect2</t>
+  </si>
+  <si>
+    <t>Barraje</t>
   </si>
 </sst>
 </file>
@@ -752,44 +755,6 @@
   </cellStyles>
   <dxfs count="41">
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -845,6 +810,44 @@
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1186,8 +1189,8 @@
     <tableColumn id="7" xr3:uid="{22F231D9-9879-4122-9BAF-253B8C04BB15}" name="regional" dataDxfId="23"/>
     <tableColumn id="2" xr3:uid="{CA56A5C1-DCFB-45F9-A91D-E19FDCFDDF4C}" name="direccion" dataDxfId="22"/>
     <tableColumn id="3" xr3:uid="{42241B89-6C4C-4F8D-8BF0-C33F36C93C1D}" name="capacidad_kva" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{56027613-F328-4A47-854A-A7351A040A78}" name="Racks" dataDxfId="0"/>
-    <tableColumn id="8" xr3:uid="{E4373386-BBF6-4449-9671-65FBEB1E22FC}" name="maximo_racks" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{56027613-F328-4A47-854A-A7351A040A78}" name="Racks" dataDxfId="20"/>
+    <tableColumn id="8" xr3:uid="{E4373386-BBF6-4449-9671-65FBEB1E22FC}" name="maximo_racks" dataDxfId="19"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1210,33 +1213,33 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F279930-8CE0-4458-A500-A4804307D033}" name="Tabla4" displayName="Tabla4" ref="A1:G95" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F279930-8CE0-4458-A500-A4804307D033}" name="Tabla4" displayName="Tabla4" ref="A1:G95" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
   <autoFilter ref="A1:G95" xr:uid="{4F279930-8CE0-4458-A500-A4804307D033}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6CBBC484-43B4-4212-8A72-72C36A0AA59A}" name="pdb_nombre" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{E0A6FC31-B215-4C57-B8C0-A8E53A5B832B}" name="fuente" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{4F3E6BCE-4115-4327-9F4D-9FE1AB222BE1}" name="posicion" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{0F488469-BA24-4436-842B-6D2F9F8F4214}" name="estado" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{DAED4AB6-F7E7-4C43-9177-F8900C29D95C}" name="capacidad" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{59F7B2D4-6A80-447C-B8ED-E0F301A44C2C}" name="corriente" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{DCE97B5A-FEBD-4BAD-9EB4-7754B346D6AB}" name="equipo_refencia" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{6CBBC484-43B4-4212-8A72-72C36A0AA59A}" name="pdb_nombre" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{E0A6FC31-B215-4C57-B8C0-A8E53A5B832B}" name="fuente" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{4F3E6BCE-4115-4327-9F4D-9FE1AB222BE1}" name="posicion" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{0F488469-BA24-4436-842B-6D2F9F8F4214}" name="estado" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{DAED4AB6-F7E7-4C43-9177-F8900C29D95C}" name="capacidad" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{59F7B2D4-6A80-447C-B8ED-E0F301A44C2C}" name="corriente" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{DCE97B5A-FEBD-4BAD-9EB4-7754B346D6AB}" name="equipo_refencia" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DE2280A1-9E4C-4DCD-BF7E-888FBA537ECA}" name="Tabla1" displayName="Tabla1" ref="A1:H13" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DE2280A1-9E4C-4DCD-BF7E-888FBA537ECA}" name="Tabla1" displayName="Tabla1" ref="A1:H13" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:H13" xr:uid="{DE2280A1-9E4C-4DCD-BF7E-888FBA537ECA}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{3AB90701-9B35-41AA-99FD-EA000C0FBAC6}" name="nombre_rack" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{552625CA-FFA9-4D0F-9AE4-8E8AA2CFD81A}" name="Label" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{4E5A4E54-6DE7-48C8-8A66-7C97E2FA04A1}" name="u_totales" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="11" xr3:uid="{BE625927-AF15-478E-87C9-1BC144738D1C}" name="Espacio" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{D32C66C7-BCD4-4610-8774-1CC22DE4F9A0}" name="u_ocupadas_listado" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{282C4EE8-ED53-4C8B-B914-B33DF7A75E4D}" name="u_libres_listado" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{D325EA4D-3855-4FB8-8337-3E9BBFFDA68B}" name="nombre_foto" dataDxfId="3" dataCellStyle="Hipervínculo"/>
-    <tableColumn id="8" xr3:uid="{94BF02C2-1F70-4B1B-94F9-F73DDBFA1E1A}" name="Detalle_rack" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{3AB90701-9B35-41AA-99FD-EA000C0FBAC6}" name="nombre_rack" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{552625CA-FFA9-4D0F-9AE4-8E8AA2CFD81A}" name="Label" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{4E5A4E54-6DE7-48C8-8A66-7C97E2FA04A1}" name="u_totales" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="11" xr3:uid="{BE625927-AF15-478E-87C9-1BC144738D1C}" name="Espacio" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{D32C66C7-BCD4-4610-8774-1CC22DE4F9A0}" name="u_ocupadas_listado" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{282C4EE8-ED53-4C8B-B914-B33DF7A75E4D}" name="u_libres_listado" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{D325EA4D-3855-4FB8-8337-3E9BBFFDA68B}" name="nombre_foto" dataDxfId="1" dataCellStyle="Hipervínculo"/>
+    <tableColumn id="8" xr3:uid="{94BF02C2-1F70-4B1B-94F9-F73DDBFA1E1A}" name="Detalle_rack" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1573,7 +1576,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>4</v>
@@ -1585,16 +1588,16 @@
         <v>8</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1608,10 +1611,10 @@
         <v>7</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>0</v>
@@ -1633,7 +1636,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70FE85F0-6249-49C0-98C3-75140ABDEF17}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -1646,32 +1649,32 @@
     <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>10</v>
@@ -1683,64 +1686,64 @@
         <v>12</v>
       </c>
       <c r="E2" s="1">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E3" s="1">
         <v>400</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>162</v>
       </c>
       <c r="E4" s="1">
         <v>400</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>13</v>
@@ -1755,16 +1758,18 @@
         <v>225</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>16</v>
+        <v>193</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>11</v>
@@ -1776,18 +1781,18 @@
         <v>125</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>17</v>
+        <v>194</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>11</v>
@@ -1799,187 +1804,196 @@
         <v>125</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E8" s="1">
         <v>500</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E9" s="1">
         <v>500</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E10" s="1">
         <v>500</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+      <c r="H10" s="1"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E11" s="1">
         <v>500</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="G11" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E12" s="1">
+        <v>250</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B12" s="1" t="s">
+      <c r="C13" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="E13" s="1">
+        <v>250</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D14" s="1" t="s">
         <v>156</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="E12" s="1">
-        <v>150</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>153</v>
-      </c>
-      <c r="E13" s="1">
-        <v>150</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="E14" s="1">
         <v>250</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="G14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E15" s="1">
         <v>250</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="G15" s="1"/>
+        <v>168</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>195</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
@@ -2005,25 +2019,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -2043,10 +2057,10 @@
         <v>80</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -2066,15 +2080,15 @@
         <v>6</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>2</v>
@@ -2089,15 +2103,15 @@
         <v>6</v>
       </c>
       <c r="F4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>2</v>
@@ -2112,15 +2126,15 @@
         <v>16</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>2</v>
@@ -2135,15 +2149,15 @@
         <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>2</v>
@@ -2161,12 +2175,12 @@
         <v>23</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>2</v>
@@ -2181,15 +2195,15 @@
         <v>100</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>2</v>
@@ -2204,15 +2218,15 @@
         <v>10</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>2</v>
@@ -2227,15 +2241,15 @@
         <v>10</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>2</v>
@@ -2250,15 +2264,15 @@
         <v>10</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>2</v>
@@ -2273,15 +2287,15 @@
         <v>10</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>2</v>
@@ -2296,15 +2310,15 @@
         <v>10</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>2</v>
@@ -2319,15 +2333,15 @@
         <v>63</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>2</v>
@@ -2342,15 +2356,15 @@
         <v>10</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>2</v>
@@ -2365,15 +2379,15 @@
         <v>10</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>2</v>
@@ -2391,12 +2405,12 @@
         <v>25</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>2</v>
@@ -2414,12 +2428,12 @@
         <v>14</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>2</v>
@@ -2434,15 +2448,15 @@
         <v>6</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>2</v>
@@ -2457,15 +2471,15 @@
         <v>6</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>2</v>
@@ -2474,7 +2488,7 @@
         <v>20</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
@@ -2483,12 +2497,12 @@
         <v>0</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>2</v>
@@ -2497,7 +2511,7 @@
         <v>21</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E22" s="1">
         <v>0</v>
@@ -2506,15 +2520,15 @@
         <v>0</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C23" s="1">
         <v>1</v>
@@ -2526,18 +2540,18 @@
         <v>80</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C24" s="1">
         <v>2</v>
@@ -2549,18 +2563,18 @@
         <v>6</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C25" s="1">
         <v>3</v>
@@ -2572,18 +2586,18 @@
         <v>6</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C26" s="1">
         <v>4</v>
@@ -2595,18 +2609,18 @@
         <v>16</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C27" s="1">
         <v>5</v>
@@ -2618,18 +2632,18 @@
         <v>16</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C28" s="1">
         <v>6</v>
@@ -2644,15 +2658,15 @@
         <v>23</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C29" s="1">
         <v>7</v>
@@ -2664,18 +2678,18 @@
         <v>100</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C30" s="1">
         <v>8</v>
@@ -2687,18 +2701,18 @@
         <v>10</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C31" s="1">
         <v>9</v>
@@ -2710,18 +2724,18 @@
         <v>10</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C32" s="1">
         <v>10</v>
@@ -2733,18 +2747,18 @@
         <v>10</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C33" s="1">
         <v>11</v>
@@ -2756,18 +2770,18 @@
         <v>10</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C34" s="1">
         <v>12</v>
@@ -2779,18 +2793,18 @@
         <v>10</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C35" s="1">
         <v>13</v>
@@ -2802,18 +2816,18 @@
         <v>63</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G35" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C36" s="1">
         <v>14</v>
@@ -2825,18 +2839,18 @@
         <v>10</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C37" s="1">
         <v>15</v>
@@ -2851,15 +2865,15 @@
         <v>0</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C38" s="1">
         <v>16</v>
@@ -2874,15 +2888,15 @@
         <v>0</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C39" s="1">
         <v>17</v>
@@ -2897,15 +2911,15 @@
         <v>0</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C40" s="1">
         <v>18</v>
@@ -2917,18 +2931,18 @@
         <v>6</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C41" s="1">
         <v>19</v>
@@ -2943,21 +2957,21 @@
         <v>14</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C42" s="1">
         <v>20</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E42" s="1">
         <v>0</v>
@@ -2966,21 +2980,21 @@
         <v>14</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C43" s="1">
         <v>21</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E43" s="1">
         <v>0</v>
@@ -2989,12 +3003,12 @@
         <v>0</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>2</v>
@@ -3012,12 +3026,12 @@
         <v>0</v>
       </c>
       <c r="G44" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>2</v>
@@ -3035,12 +3049,12 @@
         <v>0</v>
       </c>
       <c r="G45" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>2</v>
@@ -3058,12 +3072,12 @@
         <v>0</v>
       </c>
       <c r="G46" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>2</v>
@@ -3072,7 +3086,7 @@
         <v>4</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E47" s="1">
         <v>0</v>
@@ -3081,12 +3095,12 @@
         <v>0</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>2</v>
@@ -3095,7 +3109,7 @@
         <v>5</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E48" s="1">
         <v>0</v>
@@ -3104,12 +3118,12 @@
         <v>0</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>2</v>
@@ -3118,7 +3132,7 @@
         <v>6</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E49" s="1">
         <v>0</v>
@@ -3127,12 +3141,12 @@
         <v>0</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>2</v>
@@ -3141,7 +3155,7 @@
         <v>7</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E50" s="1">
         <v>0</v>
@@ -3150,12 +3164,12 @@
         <v>0</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>2</v>
@@ -3164,7 +3178,7 @@
         <v>8</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E51" s="1">
         <v>0</v>
@@ -3173,12 +3187,12 @@
         <v>0</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>2</v>
@@ -3187,7 +3201,7 @@
         <v>9</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E52" s="1">
         <v>0</v>
@@ -3196,12 +3210,12 @@
         <v>0</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>2</v>
@@ -3210,7 +3224,7 @@
         <v>10</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E53" s="1">
         <v>0</v>
@@ -3219,12 +3233,12 @@
         <v>0</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>2</v>
@@ -3233,7 +3247,7 @@
         <v>11</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E54" s="1">
         <v>0</v>
@@ -3242,12 +3256,12 @@
         <v>0</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>2</v>
@@ -3256,7 +3270,7 @@
         <v>12</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E55" s="1">
         <v>0</v>
@@ -3265,12 +3279,12 @@
         <v>0</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>2</v>
@@ -3279,7 +3293,7 @@
         <v>13</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E56" s="1">
         <v>0</v>
@@ -3288,12 +3302,12 @@
         <v>0</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>2</v>
@@ -3302,7 +3316,7 @@
         <v>14</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E57" s="1">
         <v>0</v>
@@ -3311,12 +3325,12 @@
         <v>0</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>2</v>
@@ -3325,7 +3339,7 @@
         <v>15</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E58" s="1">
         <v>0</v>
@@ -3334,12 +3348,12 @@
         <v>0</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>2</v>
@@ -3348,7 +3362,7 @@
         <v>16</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E59" s="1">
         <v>0</v>
@@ -3357,12 +3371,12 @@
         <v>0</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>2</v>
@@ -3371,7 +3385,7 @@
         <v>17</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E60" s="1">
         <v>0</v>
@@ -3380,12 +3394,12 @@
         <v>0</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>2</v>
@@ -3394,7 +3408,7 @@
         <v>18</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E61" s="1">
         <v>0</v>
@@ -3403,12 +3417,12 @@
         <v>0</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>2</v>
@@ -3417,7 +3431,7 @@
         <v>19</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E62" s="1">
         <v>0</v>
@@ -3426,12 +3440,12 @@
         <v>0</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>2</v>
@@ -3440,7 +3454,7 @@
         <v>20</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E63" s="1">
         <v>0</v>
@@ -3449,12 +3463,12 @@
         <v>0</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>2</v>
@@ -3463,7 +3477,7 @@
         <v>21</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E64" s="1">
         <v>0</v>
@@ -3472,12 +3486,12 @@
         <v>0</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>2</v>
@@ -3486,7 +3500,7 @@
         <v>22</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E65" s="1">
         <v>0</v>
@@ -3495,12 +3509,12 @@
         <v>0</v>
       </c>
       <c r="G65" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>2</v>
@@ -3509,7 +3523,7 @@
         <v>23</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E66" s="1">
         <v>0</v>
@@ -3518,12 +3532,12 @@
         <v>0</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>2</v>
@@ -3532,7 +3546,7 @@
         <v>24</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E67" s="1">
         <v>0</v>
@@ -3541,12 +3555,12 @@
         <v>0</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>2</v>
@@ -3555,7 +3569,7 @@
         <v>25</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E68" s="1">
         <v>0</v>
@@ -3564,12 +3578,12 @@
         <v>0</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>2</v>
@@ -3578,7 +3592,7 @@
         <v>26</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E69" s="1">
         <v>0</v>
@@ -3587,15 +3601,15 @@
         <v>0</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="70" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C70" s="1">
         <v>1</v>
@@ -3610,15 +3624,15 @@
         <v>0</v>
       </c>
       <c r="G70" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C71" s="1">
         <v>2</v>
@@ -3633,15 +3647,15 @@
         <v>0</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C72" s="1">
         <v>3</v>
@@ -3656,21 +3670,21 @@
         <v>0</v>
       </c>
       <c r="G72" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C73" s="1">
         <v>4</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E73" s="1">
         <v>0</v>
@@ -3679,21 +3693,21 @@
         <v>0</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C74" s="1">
         <v>5</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E74" s="1">
         <v>0</v>
@@ -3702,21 +3716,21 @@
         <v>0</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C75" s="1">
         <v>6</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E75" s="1">
         <v>0</v>
@@ -3725,21 +3739,21 @@
         <v>0</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C76" s="1">
         <v>7</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E76" s="1">
         <v>0</v>
@@ -3748,21 +3762,21 @@
         <v>0</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C77" s="1">
         <v>8</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E77" s="1">
         <v>0</v>
@@ -3771,21 +3785,21 @@
         <v>0</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C78" s="1">
         <v>9</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E78" s="1">
         <v>0</v>
@@ -3794,21 +3808,21 @@
         <v>0</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C79" s="1">
         <v>10</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E79" s="1">
         <v>0</v>
@@ -3817,21 +3831,21 @@
         <v>0</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C80" s="1">
         <v>11</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E80" s="1">
         <v>0</v>
@@ -3840,21 +3854,21 @@
         <v>0</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C81" s="1">
         <v>12</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E81" s="1">
         <v>0</v>
@@ -3863,21 +3877,21 @@
         <v>0</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C82" s="1">
         <v>13</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E82" s="1">
         <v>0</v>
@@ -3886,21 +3900,21 @@
         <v>0</v>
       </c>
       <c r="G82" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C83" s="1">
         <v>14</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E83" s="1">
         <v>0</v>
@@ -3909,21 +3923,21 @@
         <v>0</v>
       </c>
       <c r="G83" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C84" s="1">
         <v>15</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E84" s="1">
         <v>0</v>
@@ -3932,21 +3946,21 @@
         <v>0</v>
       </c>
       <c r="G84" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C85" s="1">
         <v>16</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E85" s="1">
         <v>0</v>
@@ -3955,21 +3969,21 @@
         <v>0</v>
       </c>
       <c r="G85" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C86" s="1">
         <v>17</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E86" s="1">
         <v>0</v>
@@ -3978,21 +3992,21 @@
         <v>0</v>
       </c>
       <c r="G86" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C87" s="1">
         <v>18</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E87" s="1">
         <v>0</v>
@@ -4001,21 +4015,21 @@
         <v>0</v>
       </c>
       <c r="G87" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C88" s="1">
         <v>19</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E88" s="1">
         <v>0</v>
@@ -4024,21 +4038,21 @@
         <v>0</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C89" s="1">
         <v>20</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E89" s="1">
         <v>0</v>
@@ -4047,21 +4061,21 @@
         <v>0</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C90" s="1">
         <v>21</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E90" s="1">
         <v>0</v>
@@ -4070,21 +4084,21 @@
         <v>0</v>
       </c>
       <c r="G90" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C91" s="1">
         <v>22</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E91" s="1">
         <v>0</v>
@@ -4093,21 +4107,21 @@
         <v>0</v>
       </c>
       <c r="G91" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C92" s="1">
         <v>23</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E92" s="1">
         <v>0</v>
@@ -4116,21 +4130,21 @@
         <v>0</v>
       </c>
       <c r="G92" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C93" s="1">
         <v>24</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E93" s="1">
         <v>0</v>
@@ -4139,21 +4153,21 @@
         <v>0</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C94" s="1">
         <v>25</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E94" s="1">
         <v>0</v>
@@ -4162,21 +4176,21 @@
         <v>0</v>
       </c>
       <c r="G94" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C95" s="1">
         <v>26</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E95" s="1">
         <v>0</v>
@@ -4185,7 +4199,7 @@
         <v>0</v>
       </c>
       <c r="G95" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -4214,334 +4228,334 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" t="s">
         <v>98</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="G1" t="s">
-        <v>100</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>104</v>
       </c>
       <c r="C2" s="1">
         <v>44</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C3" s="1">
         <v>45</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C4" s="1">
         <v>46</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C5" s="1">
         <v>44</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C6" s="1">
         <v>45</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C7" s="1">
         <v>45</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C8" s="1">
         <v>45</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C9" s="1">
         <v>45</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C10" s="1">
         <v>45</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C11" s="1">
         <v>45</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C12" s="1">
         <v>45</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C13" s="1">
         <v>45</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="H13" s="1"/>
     </row>

</xml_diff>